<commit_message>
Update Shopify products export - 2026-04-10 06:00:59
</commit_message>
<xml_diff>
--- a/shopify_products_export.xlsx
+++ b/shopify_products_export.xlsx
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="G12" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1101,11 +1101,11 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>31.50</t>
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>157</v>
+        <v>305</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1140,11 +1140,11 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>31.50</t>
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>317</v>
+        <v>915</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1690,7 +1690,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
@@ -1768,7 +1768,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="n">
-        <v>136</v>
+        <v>234</v>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="n">
-        <v>63</v>
+        <v>159</v>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
@@ -4030,7 +4030,7 @@
         </is>
       </c>
       <c r="G92" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
@@ -4342,7 +4342,7 @@
         </is>
       </c>
       <c r="G100" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
@@ -4420,7 +4420,7 @@
         </is>
       </c>
       <c r="G102" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
@@ -4459,7 +4459,7 @@
         </is>
       </c>
       <c r="G103" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
@@ -4654,7 +4654,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -6331,7 +6331,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6916,7 +6916,7 @@
         </is>
       </c>
       <c r="G166" s="2" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
@@ -8905,7 +8905,7 @@
         </is>
       </c>
       <c r="G217" s="2" t="n">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
@@ -9646,7 +9646,7 @@
         </is>
       </c>
       <c r="G236" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H236" s="2" t="inlineStr">
         <is>
@@ -9763,7 +9763,7 @@
         </is>
       </c>
       <c r="G239" s="2" t="n">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
@@ -9802,7 +9802,7 @@
         </is>
       </c>
       <c r="G240" s="2" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H240" s="2" t="inlineStr">
         <is>
@@ -11596,7 +11596,7 @@
         </is>
       </c>
       <c r="G286" s="2" t="n">
-        <v>1347</v>
+        <v>1338</v>
       </c>
       <c r="H286" s="2" t="inlineStr">
         <is>
@@ -11635,7 +11635,7 @@
         </is>
       </c>
       <c r="G287" s="2" t="n">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="H287" s="2" t="inlineStr">
         <is>
@@ -11674,7 +11674,7 @@
         </is>
       </c>
       <c r="G288" s="2" t="n">
-        <v>387</v>
+        <v>187</v>
       </c>
       <c r="H288" s="2" t="inlineStr">
         <is>
@@ -11713,7 +11713,7 @@
         </is>
       </c>
       <c r="G289" s="2" t="n">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="H289" s="2" t="inlineStr">
         <is>
@@ -11752,7 +11752,7 @@
         </is>
       </c>
       <c r="G290" s="2" t="n">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="H290" s="2" t="inlineStr">
         <is>
@@ -11947,7 +11947,7 @@
         </is>
       </c>
       <c r="G295" s="2" t="n">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H295" s="2" t="inlineStr">
         <is>
@@ -11986,7 +11986,7 @@
         </is>
       </c>
       <c r="G296" s="2" t="n">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="H296" s="2" t="inlineStr">
         <is>
@@ -12025,7 +12025,7 @@
         </is>
       </c>
       <c r="G297" s="2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H297" s="2" t="inlineStr">
         <is>
@@ -12532,7 +12532,7 @@
         </is>
       </c>
       <c r="G310" s="2" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="H310" s="2" t="inlineStr">
         <is>
@@ -13039,7 +13039,7 @@
         </is>
       </c>
       <c r="G323" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H323" s="2" t="inlineStr">
         <is>
@@ -13156,7 +13156,7 @@
         </is>
       </c>
       <c r="G326" s="2" t="n">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="H326" s="2" t="inlineStr">
         <is>
@@ -13585,7 +13585,7 @@
         </is>
       </c>
       <c r="G337" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H337" s="2" t="inlineStr">
         <is>
@@ -13897,7 +13897,7 @@
         </is>
       </c>
       <c r="G345" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H345" s="2" t="inlineStr">
         <is>
@@ -13975,7 +13975,7 @@
         </is>
       </c>
       <c r="G347" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H347" s="2" t="inlineStr">
         <is>
@@ -14517,11 +14517,11 @@
       <c r="E361" s="2" t="inlineStr"/>
       <c r="F361" s="2" t="inlineStr">
         <is>
-          <t>780.00</t>
+          <t>759.00</t>
         </is>
       </c>
       <c r="G361" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H361" s="2" t="inlineStr">
         <is>
@@ -14556,11 +14556,11 @@
       <c r="E362" s="2" t="inlineStr"/>
       <c r="F362" s="2" t="inlineStr">
         <is>
-          <t>780.00</t>
+          <t>759.00</t>
         </is>
       </c>
       <c r="G362" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H362" s="2" t="inlineStr">
         <is>
@@ -14595,11 +14595,11 @@
       <c r="E363" s="2" t="inlineStr"/>
       <c r="F363" s="2" t="inlineStr">
         <is>
-          <t>780.00</t>
+          <t>759.00</t>
         </is>
       </c>
       <c r="G363" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H363" s="2" t="inlineStr">
         <is>
@@ -14634,11 +14634,11 @@
       <c r="E364" s="2" t="inlineStr"/>
       <c r="F364" s="2" t="inlineStr">
         <is>
-          <t>780.00</t>
+          <t>759.00</t>
         </is>
       </c>
       <c r="G364" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H364" s="2" t="inlineStr">
         <is>
@@ -15574,7 +15574,7 @@
         </is>
       </c>
       <c r="G388" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H388" s="2" t="inlineStr">
         <is>
@@ -15652,7 +15652,7 @@
         </is>
       </c>
       <c r="G390" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H390" s="2" t="inlineStr">
         <is>
@@ -15882,11 +15882,11 @@
       <c r="E396" s="2" t="inlineStr"/>
       <c r="F396" s="2" t="inlineStr">
         <is>
-          <t>549.00</t>
+          <t>555.00</t>
         </is>
       </c>
       <c r="G396" s="2" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="H396" s="2" t="inlineStr">
         <is>
@@ -15921,11 +15921,11 @@
       <c r="E397" s="2" t="inlineStr"/>
       <c r="F397" s="2" t="inlineStr">
         <is>
-          <t>549.00</t>
+          <t>555.00</t>
         </is>
       </c>
       <c r="G397" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H397" s="2" t="inlineStr">
         <is>
@@ -15934,7 +15934,7 @@
       </c>
       <c r="I397" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -15960,11 +15960,11 @@
       <c r="E398" s="2" t="inlineStr"/>
       <c r="F398" s="2" t="inlineStr">
         <is>
-          <t>549.00</t>
+          <t>555.00</t>
         </is>
       </c>
       <c r="G398" s="2" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="H398" s="2" t="inlineStr">
         <is>
@@ -16077,11 +16077,11 @@
       <c r="E401" s="2" t="inlineStr"/>
       <c r="F401" s="2" t="inlineStr">
         <is>
-          <t>885.00</t>
+          <t>945.00</t>
         </is>
       </c>
       <c r="G401" s="2" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="H401" s="2" t="inlineStr">
         <is>
@@ -16116,11 +16116,11 @@
       <c r="E402" s="2" t="inlineStr"/>
       <c r="F402" s="2" t="inlineStr">
         <is>
-          <t>885.00</t>
+          <t>945.00</t>
         </is>
       </c>
       <c r="G402" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H402" s="2" t="inlineStr">
         <is>
@@ -16129,7 +16129,7 @@
       </c>
       <c r="I402" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -16155,11 +16155,11 @@
       <c r="E403" s="2" t="inlineStr"/>
       <c r="F403" s="2" t="inlineStr">
         <is>
-          <t>885.00</t>
+          <t>945.00</t>
         </is>
       </c>
       <c r="G403" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H403" s="2" t="inlineStr">
         <is>
@@ -16168,7 +16168,7 @@
       </c>
       <c r="I403" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -18109,7 +18109,7 @@
         </is>
       </c>
       <c r="G453" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H453" s="2" t="inlineStr">
         <is>
@@ -18889,7 +18889,7 @@
         </is>
       </c>
       <c r="G473" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H473" s="2" t="inlineStr">
         <is>
@@ -21151,7 +21151,7 @@
         </is>
       </c>
       <c r="G531" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H531" s="2" t="inlineStr">
         <is>
@@ -21190,7 +21190,7 @@
         </is>
       </c>
       <c r="G532" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H532" s="2" t="inlineStr">
         <is>
@@ -21463,7 +21463,7 @@
         </is>
       </c>
       <c r="G539" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H539" s="2" t="inlineStr">
         <is>
@@ -21472,7 +21472,7 @@
       </c>
       <c r="I539" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21502,7 +21502,7 @@
         </is>
       </c>
       <c r="G540" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H540" s="2" t="inlineStr">
         <is>
@@ -21511,7 +21511,7 @@
       </c>
       <c r="I540" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -21541,7 +21541,7 @@
         </is>
       </c>
       <c r="G541" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H541" s="2" t="inlineStr">
         <is>
@@ -21892,7 +21892,7 @@
         </is>
       </c>
       <c r="G550" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H550" s="2" t="inlineStr">
         <is>
@@ -22009,7 +22009,7 @@
         </is>
       </c>
       <c r="G553" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H553" s="2" t="inlineStr">
         <is>
@@ -22204,7 +22204,7 @@
         </is>
       </c>
       <c r="G558" s="2" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="H558" s="2" t="inlineStr">
         <is>
@@ -22243,7 +22243,7 @@
         </is>
       </c>
       <c r="G559" s="2" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H559" s="2" t="inlineStr">
         <is>
@@ -22252,7 +22252,7 @@
       </c>
       <c r="I559" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -22321,7 +22321,7 @@
         </is>
       </c>
       <c r="G561" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H561" s="2" t="inlineStr">
         <is>
@@ -22360,7 +22360,7 @@
         </is>
       </c>
       <c r="G562" s="2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H562" s="2" t="inlineStr">
         <is>
@@ -25402,7 +25402,7 @@
         </is>
       </c>
       <c r="G640" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H640" s="2" t="inlineStr">
         <is>
@@ -25411,7 +25411,7 @@
       </c>
       <c r="I640" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -25441,7 +25441,7 @@
         </is>
       </c>
       <c r="G641" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H641" s="2" t="inlineStr">
         <is>
@@ -25450,7 +25450,7 @@
       </c>
       <c r="I641" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -25480,7 +25480,7 @@
         </is>
       </c>
       <c r="G642" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H642" s="2" t="inlineStr">
         <is>
@@ -25489,7 +25489,7 @@
       </c>
       <c r="I642" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -25519,7 +25519,7 @@
         </is>
       </c>
       <c r="G643" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H643" s="2" t="inlineStr">
         <is>
@@ -26962,7 +26962,7 @@
         </is>
       </c>
       <c r="G680" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H680" s="2" t="inlineStr">
         <is>
@@ -27001,7 +27001,7 @@
         </is>
       </c>
       <c r="G681" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H681" s="2" t="inlineStr">
         <is>
@@ -27010,7 +27010,7 @@
       </c>
       <c r="I681" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -27079,7 +27079,7 @@
         </is>
       </c>
       <c r="G683" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H683" s="2" t="inlineStr">
         <is>
@@ -27088,7 +27088,7 @@
       </c>
       <c r="I683" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -30433,7 +30433,7 @@
         </is>
       </c>
       <c r="G769" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H769" s="2" t="inlineStr">
         <is>
@@ -30472,7 +30472,7 @@
         </is>
       </c>
       <c r="G770" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H770" s="2" t="inlineStr">
         <is>
@@ -30511,7 +30511,7 @@
         </is>
       </c>
       <c r="G771" s="2" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H771" s="2" t="inlineStr">
         <is>
@@ -30550,7 +30550,7 @@
         </is>
       </c>
       <c r="G772" s="2" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H772" s="2" t="inlineStr">
         <is>
@@ -31521,11 +31521,11 @@
       <c r="E797" s="2" t="inlineStr"/>
       <c r="F797" s="2" t="inlineStr">
         <is>
-          <t>2250.00</t>
+          <t>2085.00</t>
         </is>
       </c>
       <c r="G797" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H797" s="2" t="inlineStr">
         <is>
@@ -31560,11 +31560,11 @@
       <c r="E798" s="2" t="inlineStr"/>
       <c r="F798" s="2" t="inlineStr">
         <is>
-          <t>2250.00</t>
+          <t>2085.00</t>
         </is>
       </c>
       <c r="G798" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H798" s="2" t="inlineStr">
         <is>
@@ -31603,7 +31603,7 @@
         </is>
       </c>
       <c r="G799" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H799" s="2" t="inlineStr">
         <is>
@@ -31642,7 +31642,7 @@
         </is>
       </c>
       <c r="G800" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H800" s="2" t="inlineStr">
         <is>
@@ -31681,7 +31681,7 @@
         </is>
       </c>
       <c r="G801" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H801" s="2" t="inlineStr">
         <is>
@@ -32032,7 +32032,7 @@
         </is>
       </c>
       <c r="G810" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H810" s="2" t="inlineStr">
         <is>
@@ -32149,7 +32149,7 @@
         </is>
       </c>
       <c r="G813" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H813" s="2" t="inlineStr">
         <is>
@@ -32158,7 +32158,7 @@
       </c>
       <c r="I813" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -32188,7 +32188,7 @@
         </is>
       </c>
       <c r="G814" s="2" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="H814" s="2" t="inlineStr">
         <is>
@@ -32227,7 +32227,7 @@
         </is>
       </c>
       <c r="G815" s="2" t="n">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="H815" s="2" t="inlineStr">
         <is>
@@ -32266,7 +32266,7 @@
         </is>
       </c>
       <c r="G816" s="2" t="n">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="H816" s="2" t="inlineStr">
         <is>
@@ -32305,7 +32305,7 @@
         </is>
       </c>
       <c r="G817" s="2" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="H817" s="2" t="inlineStr">
         <is>
@@ -32344,7 +32344,7 @@
         </is>
       </c>
       <c r="G818" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="H818" s="2" t="inlineStr">
         <is>
@@ -32383,7 +32383,7 @@
         </is>
       </c>
       <c r="G819" s="2" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="H819" s="2" t="inlineStr">
         <is>
@@ -32422,7 +32422,7 @@
         </is>
       </c>
       <c r="G820" s="2" t="n">
-        <v>11</v>
+        <v>51</v>
       </c>
       <c r="H820" s="2" t="inlineStr">
         <is>
@@ -33085,7 +33085,7 @@
         </is>
       </c>
       <c r="G837" s="2" t="n">
-        <v>16</v>
+        <v>75</v>
       </c>
       <c r="H837" s="2" t="inlineStr">
         <is>
@@ -33124,7 +33124,7 @@
         </is>
       </c>
       <c r="G838" s="2" t="n">
-        <v>58</v>
+        <v>116</v>
       </c>
       <c r="H838" s="2" t="inlineStr">
         <is>
@@ -33163,7 +33163,7 @@
         </is>
       </c>
       <c r="G839" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H839" s="2" t="inlineStr">
         <is>
@@ -33172,7 +33172,7 @@
       </c>
       <c r="I839" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -33202,7 +33202,7 @@
         </is>
       </c>
       <c r="G840" s="2" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="H840" s="2" t="inlineStr">
         <is>
@@ -34216,7 +34216,7 @@
         </is>
       </c>
       <c r="G866" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H866" s="2" t="inlineStr">
         <is>
@@ -34368,7 +34368,7 @@
       <c r="E870" s="2" t="inlineStr"/>
       <c r="F870" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>45.00</t>
         </is>
       </c>
       <c r="G870" s="2" t="n">
@@ -34407,7 +34407,7 @@
       <c r="E871" s="2" t="inlineStr"/>
       <c r="F871" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>45.00</t>
         </is>
       </c>
       <c r="G871" s="2" t="n">
@@ -34446,7 +34446,7 @@
       <c r="E872" s="2" t="inlineStr"/>
       <c r="F872" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>45.00</t>
         </is>
       </c>
       <c r="G872" s="2" t="n">
@@ -34485,7 +34485,7 @@
       <c r="E873" s="2" t="inlineStr"/>
       <c r="F873" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>45.00</t>
         </is>
       </c>
       <c r="G873" s="2" t="n">
@@ -34524,7 +34524,7 @@
       <c r="E874" s="2" t="inlineStr"/>
       <c r="F874" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>45.00</t>
         </is>
       </c>
       <c r="G874" s="2" t="n">
@@ -34762,7 +34762,7 @@
         </is>
       </c>
       <c r="G880" s="2" t="n">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="H880" s="2" t="inlineStr">
         <is>
@@ -34801,7 +34801,7 @@
         </is>
       </c>
       <c r="G881" s="2" t="n">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="H881" s="2" t="inlineStr">
         <is>
@@ -34879,7 +34879,7 @@
         </is>
       </c>
       <c r="G883" s="2" t="n">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H883" s="2" t="inlineStr">
         <is>
@@ -35600,7 +35600,7 @@
         </is>
       </c>
       <c r="G902" s="2" t="n">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H902" s="2" t="inlineStr">
         <is>
@@ -35639,7 +35639,7 @@
         </is>
       </c>
       <c r="G903" s="2" t="n">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="H903" s="2" t="inlineStr">
         <is>
@@ -35795,7 +35795,7 @@
         </is>
       </c>
       <c r="G907" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H907" s="2" t="inlineStr">
         <is>
@@ -35990,7 +35990,7 @@
         </is>
       </c>
       <c r="G912" s="2" t="n">
-        <v>234</v>
+        <v>463</v>
       </c>
       <c r="H912" s="2" t="inlineStr">
         <is>
@@ -36068,7 +36068,7 @@
         </is>
       </c>
       <c r="G914" s="2" t="n">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="H914" s="2" t="inlineStr">
         <is>
@@ -36107,7 +36107,7 @@
         </is>
       </c>
       <c r="G915" s="2" t="n">
-        <v>871</v>
+        <v>863</v>
       </c>
       <c r="H915" s="2" t="inlineStr">
         <is>
@@ -36263,7 +36263,7 @@
         </is>
       </c>
       <c r="G919" s="2" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H919" s="2" t="inlineStr">
         <is>
@@ -36302,7 +36302,7 @@
         </is>
       </c>
       <c r="G920" s="2" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H920" s="2" t="inlineStr">
         <is>
@@ -36419,7 +36419,7 @@
         </is>
       </c>
       <c r="G923" s="2" t="n">
-        <v>203</v>
+        <v>160</v>
       </c>
       <c r="H923" s="2" t="inlineStr">
         <is>
@@ -36458,7 +36458,7 @@
         </is>
       </c>
       <c r="G924" s="2" t="n">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="H924" s="2" t="inlineStr">
         <is>
@@ -36536,7 +36536,7 @@
         </is>
       </c>
       <c r="G926" s="2" t="n">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="H926" s="2" t="inlineStr">
         <is>
@@ -36614,7 +36614,7 @@
         </is>
       </c>
       <c r="G928" s="2" t="n">
-        <v>346</v>
+        <v>327</v>
       </c>
       <c r="H928" s="2" t="inlineStr">
         <is>
@@ -36692,7 +36692,7 @@
         </is>
       </c>
       <c r="G930" s="2" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="H930" s="2" t="inlineStr">
         <is>
@@ -37043,7 +37043,7 @@
         </is>
       </c>
       <c r="G939" s="2" t="n">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H939" s="2" t="inlineStr">
         <is>
@@ -37355,7 +37355,7 @@
         </is>
       </c>
       <c r="G947" s="2" t="n">
-        <v>576</v>
+        <v>562</v>
       </c>
       <c r="H947" s="2" t="inlineStr">
         <is>
@@ -37784,7 +37784,7 @@
         </is>
       </c>
       <c r="G958" s="2" t="n">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="H958" s="2" t="inlineStr">
         <is>
@@ -37823,7 +37823,7 @@
         </is>
       </c>
       <c r="G959" s="2" t="n">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="H959" s="2" t="inlineStr">
         <is>
@@ -38291,7 +38291,7 @@
         </is>
       </c>
       <c r="G971" s="2" t="n">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H971" s="2" t="inlineStr">
         <is>
@@ -38447,7 +38447,7 @@
         </is>
       </c>
       <c r="G975" s="2" t="n">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="H975" s="2" t="inlineStr">
         <is>
@@ -38486,7 +38486,7 @@
         </is>
       </c>
       <c r="G976" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H976" s="2" t="inlineStr">
         <is>
@@ -38525,7 +38525,7 @@
         </is>
       </c>
       <c r="G977" s="2" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="H977" s="2" t="inlineStr">
         <is>
@@ -38564,7 +38564,7 @@
         </is>
       </c>
       <c r="G978" s="2" t="n">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="H978" s="2" t="inlineStr">
         <is>
@@ -38759,7 +38759,7 @@
         </is>
       </c>
       <c r="G983" s="2" t="n">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="H983" s="2" t="inlineStr">
         <is>
@@ -38989,11 +38989,11 @@
       <c r="E989" s="2" t="inlineStr"/>
       <c r="F989" s="2" t="inlineStr">
         <is>
-          <t>105.00</t>
+          <t>99.00</t>
         </is>
       </c>
       <c r="G989" s="2" t="n">
-        <v>84</v>
+        <v>134</v>
       </c>
       <c r="H989" s="2" t="inlineStr">
         <is>
@@ -39028,11 +39028,11 @@
       <c r="E990" s="2" t="inlineStr"/>
       <c r="F990" s="2" t="inlineStr">
         <is>
-          <t>105.00</t>
+          <t>99.00</t>
         </is>
       </c>
       <c r="G990" s="2" t="n">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="H990" s="2" t="inlineStr">
         <is>
@@ -39110,7 +39110,7 @@
         </is>
       </c>
       <c r="G992" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H992" s="2" t="inlineStr">
         <is>
@@ -39188,7 +39188,7 @@
         </is>
       </c>
       <c r="G994" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H994" s="2" t="inlineStr">
         <is>
@@ -39266,7 +39266,7 @@
         </is>
       </c>
       <c r="G996" s="2" t="n">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H996" s="2" t="inlineStr">
         <is>
@@ -39383,7 +39383,7 @@
         </is>
       </c>
       <c r="G999" s="2" t="n">
-        <v>424</v>
+        <v>219</v>
       </c>
       <c r="H999" s="2" t="inlineStr">
         <is>
@@ -39500,7 +39500,7 @@
         </is>
       </c>
       <c r="G1002" s="2" t="n">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H1002" s="2" t="inlineStr">
         <is>
@@ -39578,7 +39578,7 @@
         </is>
       </c>
       <c r="G1004" s="2" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="H1004" s="2" t="inlineStr">
         <is>
@@ -39812,7 +39812,7 @@
         </is>
       </c>
       <c r="G1010" s="2" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H1010" s="2" t="inlineStr">
         <is>
@@ -40046,7 +40046,7 @@
         </is>
       </c>
       <c r="G1016" s="2" t="n">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="H1016" s="2" t="inlineStr">
         <is>
@@ -40163,7 +40163,7 @@
         </is>
       </c>
       <c r="G1019" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H1019" s="2" t="inlineStr">
         <is>
@@ -40202,7 +40202,7 @@
         </is>
       </c>
       <c r="G1020" s="2" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="H1020" s="2" t="inlineStr">
         <is>
@@ -40241,7 +40241,7 @@
         </is>
       </c>
       <c r="G1021" s="2" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H1021" s="2" t="inlineStr">
         <is>
@@ -40514,7 +40514,7 @@
         </is>
       </c>
       <c r="G1028" s="2" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H1028" s="2" t="inlineStr">
         <is>
@@ -40631,7 +40631,7 @@
         </is>
       </c>
       <c r="G1031" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H1031" s="2" t="inlineStr">
         <is>
@@ -40865,7 +40865,7 @@
         </is>
       </c>
       <c r="G1037" s="2" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="H1037" s="2" t="inlineStr">
         <is>
@@ -40943,7 +40943,7 @@
         </is>
       </c>
       <c r="G1039" s="2" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H1039" s="2" t="inlineStr">
         <is>
@@ -41294,7 +41294,7 @@
         </is>
       </c>
       <c r="G1048" s="2" t="n">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H1048" s="2" t="inlineStr">
         <is>
@@ -42035,7 +42035,7 @@
         </is>
       </c>
       <c r="G1067" s="2" t="n">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H1067" s="2" t="inlineStr">
         <is>
@@ -42074,7 +42074,7 @@
         </is>
       </c>
       <c r="G1068" s="2" t="n">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="H1068" s="2" t="inlineStr">
         <is>
@@ -42152,7 +42152,7 @@
         </is>
       </c>
       <c r="G1070" s="2" t="n">
-        <v>328</v>
+        <v>314</v>
       </c>
       <c r="H1070" s="2" t="inlineStr">
         <is>
@@ -42308,7 +42308,7 @@
         </is>
       </c>
       <c r="G1074" s="2" t="n">
-        <v>918</v>
+        <v>914</v>
       </c>
       <c r="H1074" s="2" t="inlineStr">
         <is>
@@ -42659,7 +42659,7 @@
         </is>
       </c>
       <c r="G1083" s="2" t="n">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="H1083" s="2" t="inlineStr">
         <is>
@@ -43283,7 +43283,7 @@
         </is>
       </c>
       <c r="G1099" s="2" t="n">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H1099" s="2" t="inlineStr">
         <is>
@@ -43322,7 +43322,7 @@
         </is>
       </c>
       <c r="G1100" s="2" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H1100" s="2" t="inlineStr">
         <is>
@@ -44687,7 +44687,7 @@
         </is>
       </c>
       <c r="G1135" s="2" t="n">
-        <v>668</v>
+        <v>661</v>
       </c>
       <c r="H1135" s="2" t="inlineStr">
         <is>
@@ -44726,7 +44726,7 @@
         </is>
       </c>
       <c r="G1136" s="2" t="n">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H1136" s="2" t="inlineStr">
         <is>
@@ -45584,7 +45584,7 @@
         </is>
       </c>
       <c r="G1158" s="2" t="n">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H1158" s="2" t="inlineStr">
         <is>
@@ -45623,7 +45623,7 @@
         </is>
       </c>
       <c r="G1159" s="2" t="n">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="H1159" s="2" t="inlineStr">
         <is>
@@ -45658,11 +45658,11 @@
       <c r="E1160" s="2" t="inlineStr"/>
       <c r="F1160" s="2" t="inlineStr">
         <is>
-          <t>75.00</t>
+          <t>66.00</t>
         </is>
       </c>
       <c r="G1160" s="2" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H1160" s="2" t="inlineStr">
         <is>
@@ -45671,7 +45671,7 @@
       </c>
       <c r="I1160" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -45697,11 +45697,11 @@
       <c r="E1161" s="2" t="inlineStr"/>
       <c r="F1161" s="2" t="inlineStr">
         <is>
-          <t>75.00</t>
+          <t>66.00</t>
         </is>
       </c>
       <c r="G1161" s="2" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="H1161" s="2" t="inlineStr">
         <is>
@@ -46871,7 +46871,7 @@
         </is>
       </c>
       <c r="G1191" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H1191" s="2" t="inlineStr">
         <is>
@@ -46949,7 +46949,7 @@
         </is>
       </c>
       <c r="G1193" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H1193" s="2" t="inlineStr">
         <is>
@@ -48197,7 +48197,7 @@
         </is>
       </c>
       <c r="G1225" s="2" t="n">
-        <v>3</v>
+        <v>42</v>
       </c>
       <c r="H1225" s="2" t="inlineStr">
         <is>
@@ -49055,7 +49055,7 @@
         </is>
       </c>
       <c r="G1247" s="2" t="n">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="H1247" s="2" t="inlineStr">
         <is>
@@ -49211,7 +49211,7 @@
         </is>
       </c>
       <c r="G1251" s="2" t="n">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="H1251" s="2" t="inlineStr">
         <is>
@@ -49250,7 +49250,7 @@
         </is>
       </c>
       <c r="G1252" s="2" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H1252" s="2" t="inlineStr">
         <is>
@@ -49562,7 +49562,7 @@
         </is>
       </c>
       <c r="G1260" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H1260" s="2" t="inlineStr">
         <is>
@@ -49913,7 +49913,7 @@
         </is>
       </c>
       <c r="G1269" s="2" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H1269" s="2" t="inlineStr">
         <is>
@@ -50147,7 +50147,7 @@
         </is>
       </c>
       <c r="G1275" s="2" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H1275" s="2" t="inlineStr">
         <is>
@@ -51044,7 +51044,7 @@
         </is>
       </c>
       <c r="G1298" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H1298" s="2" t="inlineStr">
         <is>
@@ -51161,7 +51161,7 @@
         </is>
       </c>
       <c r="G1301" s="2" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H1301" s="2" t="inlineStr">
         <is>
@@ -51434,7 +51434,7 @@
         </is>
       </c>
       <c r="G1308" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H1308" s="2" t="inlineStr">
         <is>
@@ -51473,7 +51473,7 @@
         </is>
       </c>
       <c r="G1309" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H1309" s="2" t="inlineStr">
         <is>
@@ -51512,7 +51512,7 @@
         </is>
       </c>
       <c r="G1310" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H1310" s="2" t="inlineStr">
         <is>
@@ -51785,7 +51785,7 @@
         </is>
       </c>
       <c r="G1317" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H1317" s="2" t="inlineStr">
         <is>
@@ -51824,7 +51824,7 @@
         </is>
       </c>
       <c r="G1318" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H1318" s="2" t="inlineStr">
         <is>
@@ -51863,7 +51863,7 @@
         </is>
       </c>
       <c r="G1319" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H1319" s="2" t="inlineStr">
         <is>
@@ -51902,7 +51902,7 @@
         </is>
       </c>
       <c r="G1320" s="2" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H1320" s="2" t="inlineStr">
         <is>
@@ -51980,7 +51980,7 @@
         </is>
       </c>
       <c r="G1322" s="2" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H1322" s="2" t="inlineStr">
         <is>
@@ -52019,7 +52019,7 @@
         </is>
       </c>
       <c r="G1323" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H1323" s="2" t="inlineStr">
         <is>
@@ -52214,7 +52214,7 @@
         </is>
       </c>
       <c r="G1328" s="2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H1328" s="2" t="inlineStr">
         <is>
@@ -52292,7 +52292,7 @@
         </is>
       </c>
       <c r="G1330" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H1330" s="2" t="inlineStr">
         <is>
@@ -52370,7 +52370,7 @@
         </is>
       </c>
       <c r="G1332" s="2" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H1332" s="2" t="inlineStr">
         <is>
@@ -52409,7 +52409,7 @@
         </is>
       </c>
       <c r="G1333" s="2" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="H1333" s="2" t="inlineStr">
         <is>
@@ -52799,7 +52799,7 @@
         </is>
       </c>
       <c r="G1343" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H1343" s="2" t="inlineStr">
         <is>
@@ -53618,7 +53618,7 @@
         </is>
       </c>
       <c r="G1364" s="2" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H1364" s="2" t="inlineStr">
         <is>
@@ -53653,11 +53653,11 @@
       <c r="E1365" s="2" t="inlineStr"/>
       <c r="F1365" s="2" t="inlineStr">
         <is>
-          <t>195.00</t>
+          <t>210.00</t>
         </is>
       </c>
       <c r="G1365" s="2" t="n">
-        <v>42</v>
+        <v>94</v>
       </c>
       <c r="H1365" s="2" t="inlineStr">
         <is>
@@ -53891,7 +53891,7 @@
         </is>
       </c>
       <c r="G1371" s="2" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="H1371" s="2" t="inlineStr">
         <is>
@@ -54086,16 +54086,16 @@
         </is>
       </c>
       <c r="G1376" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1376" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I1376" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -54461,7 +54461,7 @@
       </c>
       <c r="C1386" s="2" t="inlineStr">
         <is>
-          <t>BYY</t>
+          <t>Moreka</t>
         </is>
       </c>
       <c r="D1386" s="2" t="inlineStr">
@@ -54500,7 +54500,7 @@
       </c>
       <c r="C1387" s="2" t="inlineStr">
         <is>
-          <t>BYY</t>
+          <t>Moreka</t>
         </is>
       </c>
       <c r="D1387" s="2" t="inlineStr">
@@ -54515,7 +54515,7 @@
         </is>
       </c>
       <c r="G1387" s="2" t="n">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H1387" s="2" t="inlineStr">
         <is>
@@ -54788,7 +54788,7 @@
         </is>
       </c>
       <c r="G1394" s="2" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H1394" s="2" t="inlineStr">
         <is>
@@ -54944,7 +54944,7 @@
         </is>
       </c>
       <c r="G1398" s="2" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H1398" s="2" t="inlineStr">
         <is>
@@ -54983,7 +54983,7 @@
         </is>
       </c>
       <c r="G1399" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H1399" s="2" t="inlineStr">
         <is>
@@ -55022,7 +55022,7 @@
         </is>
       </c>
       <c r="G1400" s="2" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H1400" s="2" t="inlineStr">
         <is>
@@ -55802,7 +55802,7 @@
         </is>
       </c>
       <c r="G1420" s="2" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H1420" s="2" t="inlineStr">
         <is>
@@ -55841,7 +55841,7 @@
         </is>
       </c>
       <c r="G1421" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H1421" s="2" t="inlineStr">
         <is>
@@ -56270,7 +56270,7 @@
         </is>
       </c>
       <c r="G1432" s="2" t="n">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="H1432" s="2" t="inlineStr">
         <is>
@@ -56309,7 +56309,7 @@
         </is>
       </c>
       <c r="G1433" s="2" t="n">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="H1433" s="2" t="inlineStr">
         <is>
@@ -56699,7 +56699,7 @@
         </is>
       </c>
       <c r="G1443" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H1443" s="2" t="inlineStr">
         <is>
@@ -56777,7 +56777,7 @@
         </is>
       </c>
       <c r="G1445" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H1445" s="2" t="inlineStr">
         <is>
@@ -58021,11 +58021,11 @@
       <c r="E1477" s="2" t="inlineStr"/>
       <c r="F1477" s="2" t="inlineStr">
         <is>
-          <t>504.00</t>
+          <t>508.50</t>
         </is>
       </c>
       <c r="G1477" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H1477" s="2" t="inlineStr">
         <is>
@@ -58060,11 +58060,11 @@
       <c r="E1478" s="2" t="inlineStr"/>
       <c r="F1478" s="2" t="inlineStr">
         <is>
-          <t>504.00</t>
+          <t>508.50</t>
         </is>
       </c>
       <c r="G1478" s="2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H1478" s="2" t="inlineStr">
         <is>
@@ -58103,7 +58103,7 @@
         </is>
       </c>
       <c r="G1479" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H1479" s="2" t="inlineStr">
         <is>
@@ -58571,7 +58571,7 @@
         </is>
       </c>
       <c r="G1491" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H1491" s="2" t="inlineStr">
         <is>
@@ -58649,7 +58649,7 @@
         </is>
       </c>
       <c r="G1493" s="2" t="n">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="H1493" s="2" t="inlineStr">
         <is>
@@ -58688,7 +58688,7 @@
         </is>
       </c>
       <c r="G1494" s="2" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="H1494" s="2" t="inlineStr">
         <is>
@@ -58727,7 +58727,7 @@
         </is>
       </c>
       <c r="G1495" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H1495" s="2" t="inlineStr">
         <is>
@@ -58736,7 +58736,7 @@
       </c>
       <c r="I1495" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -58766,7 +58766,7 @@
         </is>
       </c>
       <c r="G1496" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H1496" s="2" t="inlineStr">
         <is>
@@ -58775,7 +58775,7 @@
       </c>
       <c r="I1496" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -58879,7 +58879,7 @@
       <c r="E1499" s="2" t="inlineStr"/>
       <c r="F1499" s="2" t="inlineStr">
         <is>
-          <t>225.00</t>
+          <t>204.00</t>
         </is>
       </c>
       <c r="G1499" s="2" t="n">
@@ -58918,7 +58918,7 @@
       <c r="E1500" s="2" t="inlineStr"/>
       <c r="F1500" s="2" t="inlineStr">
         <is>
-          <t>225.00</t>
+          <t>204.00</t>
         </is>
       </c>
       <c r="G1500" s="2" t="n">
@@ -58957,11 +58957,11 @@
       <c r="E1501" s="2" t="inlineStr"/>
       <c r="F1501" s="2" t="inlineStr">
         <is>
-          <t>225.00</t>
+          <t>204.00</t>
         </is>
       </c>
       <c r="G1501" s="2" t="n">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="H1501" s="2" t="inlineStr">
         <is>
@@ -58996,11 +58996,11 @@
       <c r="E1502" s="2" t="inlineStr"/>
       <c r="F1502" s="2" t="inlineStr">
         <is>
-          <t>225.00</t>
+          <t>204.00</t>
         </is>
       </c>
       <c r="G1502" s="2" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="H1502" s="2" t="inlineStr">
         <is>
@@ -59819,7 +59819,7 @@
         </is>
       </c>
       <c r="G1523" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H1523" s="2" t="inlineStr">
         <is>
@@ -59858,7 +59858,7 @@
         </is>
       </c>
       <c r="G1524" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H1524" s="2" t="inlineStr">
         <is>
@@ -60209,7 +60209,7 @@
         </is>
       </c>
       <c r="G1533" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H1533" s="2" t="inlineStr">
         <is>
@@ -60560,7 +60560,7 @@
         </is>
       </c>
       <c r="G1542" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H1542" s="2" t="inlineStr">
         <is>
@@ -61769,7 +61769,7 @@
         </is>
       </c>
       <c r="G1573" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H1573" s="2" t="inlineStr">
         <is>
@@ -65708,7 +65708,7 @@
         </is>
       </c>
       <c r="G1674" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H1674" s="2" t="inlineStr">
         <is>
@@ -65864,7 +65864,7 @@
         </is>
       </c>
       <c r="G1678" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H1678" s="2" t="inlineStr">
         <is>
@@ -65903,7 +65903,7 @@
         </is>
       </c>
       <c r="G1679" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H1679" s="2" t="inlineStr">
         <is>
@@ -65981,7 +65981,7 @@
         </is>
       </c>
       <c r="G1681" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H1681" s="2" t="inlineStr">
         <is>
@@ -66098,16 +66098,16 @@
         </is>
       </c>
       <c r="G1684" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H1684" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I1684" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -66141,7 +66141,7 @@
       </c>
       <c r="H1685" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I1685" s="2" t="inlineStr">
@@ -66180,7 +66180,7 @@
       </c>
       <c r="H1686" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I1686" s="2" t="inlineStr">
@@ -67736,16 +67736,16 @@
         </is>
       </c>
       <c r="G1726" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1726" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I1726" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -67775,7 +67775,7 @@
         </is>
       </c>
       <c r="G1727" s="2" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H1727" s="2" t="inlineStr">
         <is>
@@ -67814,7 +67814,7 @@
         </is>
       </c>
       <c r="G1728" s="2" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H1728" s="2" t="inlineStr">
         <is>
@@ -67931,7 +67931,7 @@
         </is>
       </c>
       <c r="G1731" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H1731" s="2" t="inlineStr">
         <is>
@@ -67970,7 +67970,7 @@
         </is>
       </c>
       <c r="G1732" s="2" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H1732" s="2" t="inlineStr">
         <is>
@@ -68087,7 +68087,7 @@
         </is>
       </c>
       <c r="G1735" s="2" t="n">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="H1735" s="2" t="inlineStr">
         <is>
@@ -68165,7 +68165,7 @@
         </is>
       </c>
       <c r="G1737" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H1737" s="2" t="inlineStr">
         <is>
@@ -68243,7 +68243,7 @@
         </is>
       </c>
       <c r="G1739" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H1739" s="2" t="inlineStr">
         <is>
@@ -68282,7 +68282,7 @@
         </is>
       </c>
       <c r="G1740" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H1740" s="2" t="inlineStr">
         <is>
@@ -68438,7 +68438,7 @@
         </is>
       </c>
       <c r="G1744" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H1744" s="2" t="inlineStr">
         <is>
@@ -68477,7 +68477,7 @@
         </is>
       </c>
       <c r="G1745" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H1745" s="2" t="inlineStr">
         <is>
@@ -70466,7 +70466,7 @@
         </is>
       </c>
       <c r="G1796" s="2" t="n">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="H1796" s="2" t="inlineStr">
         <is>
@@ -70505,7 +70505,7 @@
         </is>
       </c>
       <c r="G1797" s="2" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H1797" s="2" t="inlineStr">
         <is>
@@ -70739,7 +70739,7 @@
         </is>
       </c>
       <c r="G1803" s="2" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="H1803" s="2" t="inlineStr">
         <is>
@@ -70748,7 +70748,7 @@
       </c>
       <c r="I1803" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -70856,7 +70856,7 @@
         </is>
       </c>
       <c r="G1806" s="2" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H1806" s="2" t="inlineStr">
         <is>
@@ -71909,7 +71909,7 @@
         </is>
       </c>
       <c r="G1833" s="2" t="n">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="H1833" s="2" t="inlineStr">
         <is>
@@ -73001,7 +73001,7 @@
         </is>
       </c>
       <c r="G1861" s="2" t="n">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="H1861" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update Shopify products export - 2026-05-07 06:00:59
</commit_message>
<xml_diff>
--- a/shopify_products_export.xlsx
+++ b/shopify_products_export.xlsx
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="G7" s="2" t="n">
-        <v>506</v>
+        <v>494</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -754,7 +754,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
@@ -871,7 +871,7 @@
         </is>
       </c>
       <c r="G11" s="2" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="n">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="G16" s="2" t="n">
-        <v>773</v>
+        <v>763</v>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="G17" s="2" t="n">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="n">
-        <v>599</v>
+        <v>594</v>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
@@ -1222,7 +1222,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="G31" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="n">
-        <v>233</v>
+        <v>193</v>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="n">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="n">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
@@ -2236,7 +2236,7 @@
         </is>
       </c>
       <c r="G46" s="2" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="G48" s="2" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
@@ -2353,7 +2353,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="n">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         </is>
       </c>
       <c r="G84" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
@@ -4576,7 +4576,7 @@
         </is>
       </c>
       <c r="G106" s="2" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
@@ -4654,7 +4654,7 @@
         </is>
       </c>
       <c r="G108" s="2" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
@@ -4732,7 +4732,7 @@
         </is>
       </c>
       <c r="G110" s="2" t="n">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
@@ -4810,7 +4810,7 @@
         </is>
       </c>
       <c r="G112" s="2" t="n">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
@@ -4966,7 +4966,7 @@
         </is>
       </c>
       <c r="G116" s="2" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
@@ -5005,7 +5005,7 @@
         </is>
       </c>
       <c r="G117" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
@@ -5083,7 +5083,7 @@
         </is>
       </c>
       <c r="G119" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
         </is>
       </c>
       <c r="G121" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
@@ -5629,7 +5629,7 @@
         </is>
       </c>
       <c r="G133" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
@@ -6331,7 +6331,7 @@
         </is>
       </c>
       <c r="G151" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
@@ -6370,7 +6370,7 @@
         </is>
       </c>
       <c r="G152" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
@@ -6487,7 +6487,7 @@
         </is>
       </c>
       <c r="G155" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I160" s="2" t="inlineStr">
@@ -6721,16 +6721,16 @@
         </is>
       </c>
       <c r="G161" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -6764,7 +6764,7 @@
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I162" s="2" t="inlineStr">
@@ -6799,7 +6799,7 @@
         </is>
       </c>
       <c r="G163" s="2" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
@@ -7380,11 +7380,11 @@
       <c r="E178" s="2" t="inlineStr"/>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>384.00</t>
+          <t>339.00</t>
         </is>
       </c>
       <c r="G178" s="2" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
@@ -7419,11 +7419,11 @@
       <c r="E179" s="2" t="inlineStr"/>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>384.00</t>
+          <t>339.00</t>
         </is>
       </c>
       <c r="G179" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
@@ -8437,7 +8437,7 @@
         </is>
       </c>
       <c r="G205" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -9412,7 +9412,7 @@
         </is>
       </c>
       <c r="G230" s="2" t="n">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="H230" s="2" t="inlineStr">
         <is>
@@ -9451,7 +9451,7 @@
         </is>
       </c>
       <c r="G231" s="2" t="n">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
@@ -10192,7 +10192,7 @@
         </is>
       </c>
       <c r="G250" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
@@ -10309,7 +10309,7 @@
         </is>
       </c>
       <c r="G253" s="2" t="n">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="H253" s="2" t="inlineStr">
         <is>
@@ -10348,7 +10348,7 @@
         </is>
       </c>
       <c r="G254" s="2" t="n">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="H254" s="2" t="inlineStr">
         <is>
@@ -10387,7 +10387,7 @@
         </is>
       </c>
       <c r="G255" s="2" t="n">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
@@ -10426,7 +10426,7 @@
         </is>
       </c>
       <c r="G256" s="2" t="n">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
@@ -10504,7 +10504,7 @@
         </is>
       </c>
       <c r="G258" s="2" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
@@ -12259,7 +12259,7 @@
         </is>
       </c>
       <c r="G303" s="2" t="n">
-        <v>340</v>
+        <v>687</v>
       </c>
       <c r="H303" s="2" t="inlineStr">
         <is>
@@ -12298,7 +12298,7 @@
         </is>
       </c>
       <c r="G304" s="2" t="n">
-        <v>1289</v>
+        <v>1287</v>
       </c>
       <c r="H304" s="2" t="inlineStr">
         <is>
@@ -12337,7 +12337,7 @@
         </is>
       </c>
       <c r="G305" s="2" t="n">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="H305" s="2" t="inlineStr">
         <is>
@@ -12376,7 +12376,7 @@
         </is>
       </c>
       <c r="G306" s="2" t="n">
-        <v>401</v>
+        <v>373</v>
       </c>
       <c r="H306" s="2" t="inlineStr">
         <is>
@@ -12649,7 +12649,7 @@
         </is>
       </c>
       <c r="G313" s="2" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H313" s="2" t="inlineStr">
         <is>
@@ -12688,7 +12688,7 @@
         </is>
       </c>
       <c r="G314" s="2" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H314" s="2" t="inlineStr">
         <is>
@@ -12805,7 +12805,7 @@
         </is>
       </c>
       <c r="G317" s="2" t="n">
-        <v>493</v>
+        <v>439</v>
       </c>
       <c r="H317" s="2" t="inlineStr">
         <is>
@@ -12883,7 +12883,7 @@
         </is>
       </c>
       <c r="G319" s="2" t="n">
-        <v>340</v>
+        <v>687</v>
       </c>
       <c r="H319" s="2" t="inlineStr">
         <is>
@@ -13195,7 +13195,7 @@
         </is>
       </c>
       <c r="G327" s="2" t="n">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="H327" s="2" t="inlineStr">
         <is>
@@ -13273,7 +13273,7 @@
         </is>
       </c>
       <c r="G329" s="2" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H329" s="2" t="inlineStr">
         <is>
@@ -13312,7 +13312,7 @@
         </is>
       </c>
       <c r="G330" s="2" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="H330" s="2" t="inlineStr">
         <is>
@@ -13351,7 +13351,7 @@
         </is>
       </c>
       <c r="G331" s="2" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H331" s="2" t="inlineStr">
         <is>
@@ -13858,7 +13858,7 @@
         </is>
       </c>
       <c r="G344" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="H344" s="2" t="inlineStr">
         <is>
@@ -13897,7 +13897,7 @@
         </is>
       </c>
       <c r="G345" s="2" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="H345" s="2" t="inlineStr">
         <is>
@@ -13936,7 +13936,7 @@
         </is>
       </c>
       <c r="G346" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H346" s="2" t="inlineStr">
         <is>
@@ -14131,7 +14131,7 @@
         </is>
       </c>
       <c r="G351" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H351" s="2" t="inlineStr">
         <is>
@@ -14170,7 +14170,7 @@
         </is>
       </c>
       <c r="G352" s="2" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H352" s="2" t="inlineStr">
         <is>
@@ -14365,7 +14365,7 @@
         </is>
       </c>
       <c r="G357" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H357" s="2" t="inlineStr">
         <is>
@@ -15496,7 +15496,7 @@
         </is>
       </c>
       <c r="G386" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H386" s="2" t="inlineStr">
         <is>
@@ -19006,7 +19006,7 @@
         </is>
       </c>
       <c r="G476" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H476" s="2" t="inlineStr">
         <is>
@@ -19630,7 +19630,7 @@
         </is>
       </c>
       <c r="G492" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H492" s="2" t="inlineStr">
         <is>
@@ -22048,7 +22048,7 @@
         </is>
       </c>
       <c r="G554" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H554" s="2" t="inlineStr">
         <is>
@@ -22165,7 +22165,7 @@
         </is>
       </c>
       <c r="G557" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H557" s="2" t="inlineStr">
         <is>
@@ -23257,7 +23257,7 @@
         </is>
       </c>
       <c r="G585" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H585" s="2" t="inlineStr">
         <is>
@@ -23335,7 +23335,7 @@
         </is>
       </c>
       <c r="G587" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H587" s="2" t="inlineStr">
         <is>
@@ -23413,7 +23413,7 @@
         </is>
       </c>
       <c r="G589" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H589" s="2" t="inlineStr">
         <is>
@@ -23530,7 +23530,7 @@
         </is>
       </c>
       <c r="G592" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H592" s="2" t="inlineStr">
         <is>
@@ -23920,7 +23920,7 @@
         </is>
       </c>
       <c r="G602" s="2" t="n">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="H602" s="2" t="inlineStr">
         <is>
@@ -23959,7 +23959,7 @@
         </is>
       </c>
       <c r="G603" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H603" s="2" t="inlineStr">
         <is>
@@ -24115,7 +24115,7 @@
         </is>
       </c>
       <c r="G607" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H607" s="2" t="inlineStr">
         <is>
@@ -25831,7 +25831,7 @@
         </is>
       </c>
       <c r="G651" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H651" s="2" t="inlineStr">
         <is>
@@ -26299,7 +26299,7 @@
         </is>
       </c>
       <c r="G663" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H663" s="2" t="inlineStr">
         <is>
@@ -26767,7 +26767,7 @@
         </is>
       </c>
       <c r="G675" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H675" s="2" t="inlineStr">
         <is>
@@ -27430,7 +27430,7 @@
         </is>
       </c>
       <c r="G692" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H692" s="2" t="inlineStr">
         <is>
@@ -27439,7 +27439,7 @@
       </c>
       <c r="I692" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -27547,7 +27547,7 @@
         </is>
       </c>
       <c r="G695" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H695" s="2" t="inlineStr">
         <is>
@@ -27703,7 +27703,7 @@
         </is>
       </c>
       <c r="G699" s="2" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H699" s="2" t="inlineStr">
         <is>
@@ -27859,7 +27859,7 @@
         </is>
       </c>
       <c r="G703" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H703" s="2" t="inlineStr">
         <is>
@@ -28054,7 +28054,7 @@
         </is>
       </c>
       <c r="G708" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H708" s="2" t="inlineStr">
         <is>
@@ -30004,7 +30004,7 @@
         </is>
       </c>
       <c r="G758" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H758" s="2" t="inlineStr">
         <is>
@@ -30082,7 +30082,7 @@
         </is>
       </c>
       <c r="G760" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H760" s="2" t="inlineStr">
         <is>
@@ -31681,7 +31681,7 @@
         </is>
       </c>
       <c r="G801" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H801" s="2" t="inlineStr">
         <is>
@@ -31720,7 +31720,7 @@
         </is>
       </c>
       <c r="G802" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H802" s="2" t="inlineStr">
         <is>
@@ -31759,7 +31759,7 @@
         </is>
       </c>
       <c r="G803" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H803" s="2" t="inlineStr">
         <is>
@@ -32773,7 +32773,7 @@
         </is>
       </c>
       <c r="G829" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H829" s="2" t="inlineStr">
         <is>
@@ -33007,7 +33007,7 @@
         </is>
       </c>
       <c r="G835" s="2" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H835" s="2" t="inlineStr">
         <is>
@@ -33046,7 +33046,7 @@
         </is>
       </c>
       <c r="G836" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H836" s="2" t="inlineStr">
         <is>
@@ -33397,7 +33397,7 @@
         </is>
       </c>
       <c r="G845" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H845" s="2" t="inlineStr">
         <is>
@@ -33436,7 +33436,7 @@
         </is>
       </c>
       <c r="G846" s="2" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H846" s="2" t="inlineStr">
         <is>
@@ -33475,7 +33475,7 @@
         </is>
       </c>
       <c r="G847" s="2" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="H847" s="2" t="inlineStr">
         <is>
@@ -33514,7 +33514,7 @@
         </is>
       </c>
       <c r="G848" s="2" t="n">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="H848" s="2" t="inlineStr">
         <is>
@@ -33553,7 +33553,7 @@
         </is>
       </c>
       <c r="G849" s="2" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="H849" s="2" t="inlineStr">
         <is>
@@ -33592,7 +33592,7 @@
         </is>
       </c>
       <c r="G850" s="2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="H850" s="2" t="inlineStr">
         <is>
@@ -33631,7 +33631,7 @@
         </is>
       </c>
       <c r="G851" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H851" s="2" t="inlineStr">
         <is>
@@ -33640,7 +33640,7 @@
       </c>
       <c r="I851" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -34372,7 +34372,7 @@
         </is>
       </c>
       <c r="G870" s="2" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H870" s="2" t="inlineStr">
         <is>
@@ -34528,7 +34528,7 @@
         </is>
       </c>
       <c r="G874" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H874" s="2" t="inlineStr">
         <is>
@@ -35347,7 +35347,7 @@
         </is>
       </c>
       <c r="G895" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H895" s="2" t="inlineStr">
         <is>
@@ -35542,7 +35542,7 @@
         </is>
       </c>
       <c r="G900" s="2" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="H900" s="2" t="inlineStr">
         <is>
@@ -35581,7 +35581,7 @@
         </is>
       </c>
       <c r="G901" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H901" s="2" t="inlineStr">
         <is>
@@ -36010,7 +36010,7 @@
         </is>
       </c>
       <c r="G912" s="2" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="H912" s="2" t="inlineStr">
         <is>
@@ -36123,11 +36123,11 @@
       <c r="E915" s="2" t="inlineStr"/>
       <c r="F915" s="2" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>25.50</t>
         </is>
       </c>
       <c r="G915" s="2" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="H915" s="2" t="inlineStr">
         <is>
@@ -36136,7 +36136,7 @@
       </c>
       <c r="I915" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -36162,7 +36162,7 @@
       <c r="E916" s="2" t="inlineStr"/>
       <c r="F916" s="2" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>25.50</t>
         </is>
       </c>
       <c r="G916" s="2" t="n">
@@ -36201,7 +36201,7 @@
       <c r="E917" s="2" t="inlineStr"/>
       <c r="F917" s="2" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>25.50</t>
         </is>
       </c>
       <c r="G917" s="2" t="n">
@@ -36240,7 +36240,7 @@
       <c r="E918" s="2" t="inlineStr"/>
       <c r="F918" s="2" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>25.50</t>
         </is>
       </c>
       <c r="G918" s="2" t="n">
@@ -36279,7 +36279,7 @@
       <c r="E919" s="2" t="inlineStr"/>
       <c r="F919" s="2" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>25.50</t>
         </is>
       </c>
       <c r="G919" s="2" t="n">
@@ -36318,7 +36318,7 @@
       <c r="E920" s="2" t="inlineStr"/>
       <c r="F920" s="2" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>25.50</t>
         </is>
       </c>
       <c r="G920" s="2" t="n">
@@ -36357,7 +36357,7 @@
       <c r="E921" s="2" t="inlineStr"/>
       <c r="F921" s="2" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>25.50</t>
         </is>
       </c>
       <c r="G921" s="2" t="n">
@@ -36809,7 +36809,7 @@
         </is>
       </c>
       <c r="G933" s="2" t="n">
-        <v>151</v>
+        <v>112</v>
       </c>
       <c r="H933" s="2" t="inlineStr">
         <is>
@@ -36848,7 +36848,7 @@
         </is>
       </c>
       <c r="G934" s="2" t="n">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="H934" s="2" t="inlineStr">
         <is>
@@ -36965,7 +36965,7 @@
         </is>
       </c>
       <c r="G937" s="2" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="H937" s="2" t="inlineStr">
         <is>
@@ -37004,7 +37004,7 @@
         </is>
       </c>
       <c r="G938" s="2" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="H938" s="2" t="inlineStr">
         <is>
@@ -37043,7 +37043,7 @@
         </is>
       </c>
       <c r="G939" s="2" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="H939" s="2" t="inlineStr">
         <is>
@@ -37234,11 +37234,11 @@
       <c r="E944" s="2" t="inlineStr"/>
       <c r="F944" s="2" t="inlineStr">
         <is>
-          <t>33.00</t>
+          <t>30.00</t>
         </is>
       </c>
       <c r="G944" s="2" t="n">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="H944" s="2" t="inlineStr">
         <is>
@@ -37277,7 +37277,7 @@
         </is>
       </c>
       <c r="G945" s="2" t="n">
-        <v>400</v>
+        <v>392</v>
       </c>
       <c r="H945" s="2" t="inlineStr">
         <is>
@@ -37316,7 +37316,7 @@
         </is>
       </c>
       <c r="G946" s="2" t="n">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="H946" s="2" t="inlineStr">
         <is>
@@ -37355,7 +37355,7 @@
         </is>
       </c>
       <c r="G947" s="2" t="n">
-        <v>989</v>
+        <v>942</v>
       </c>
       <c r="H947" s="2" t="inlineStr">
         <is>
@@ -37589,7 +37589,7 @@
         </is>
       </c>
       <c r="G953" s="2" t="n">
-        <v>66</v>
+        <v>44</v>
       </c>
       <c r="H953" s="2" t="inlineStr">
         <is>
@@ -37745,7 +37745,7 @@
         </is>
       </c>
       <c r="G957" s="2" t="n">
-        <v>564</v>
+        <v>539</v>
       </c>
       <c r="H957" s="2" t="inlineStr">
         <is>
@@ -37784,7 +37784,7 @@
         </is>
       </c>
       <c r="G958" s="2" t="n">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="H958" s="2" t="inlineStr">
         <is>
@@ -37858,11 +37858,11 @@
       <c r="E960" s="2" t="inlineStr"/>
       <c r="F960" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>28.50</t>
         </is>
       </c>
       <c r="G960" s="2" t="n">
-        <v>67</v>
+        <v>347</v>
       </c>
       <c r="H960" s="2" t="inlineStr">
         <is>
@@ -37940,7 +37940,7 @@
         </is>
       </c>
       <c r="G962" s="2" t="n">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H962" s="2" t="inlineStr">
         <is>
@@ -38018,7 +38018,7 @@
         </is>
       </c>
       <c r="G964" s="2" t="n">
-        <v>109</v>
+        <v>509</v>
       </c>
       <c r="H964" s="2" t="inlineStr">
         <is>
@@ -38057,7 +38057,7 @@
         </is>
       </c>
       <c r="G965" s="2" t="n">
-        <v>23</v>
+        <v>203</v>
       </c>
       <c r="H965" s="2" t="inlineStr">
         <is>
@@ -38131,11 +38131,11 @@
       <c r="E967" s="2" t="inlineStr"/>
       <c r="F967" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>33.00</t>
         </is>
       </c>
       <c r="G967" s="2" t="n">
-        <v>255</v>
+        <v>459</v>
       </c>
       <c r="H967" s="2" t="inlineStr">
         <is>
@@ -38170,11 +38170,11 @@
       <c r="E968" s="2" t="inlineStr"/>
       <c r="F968" s="2" t="inlineStr">
         <is>
-          <t>30.00</t>
+          <t>33.00</t>
         </is>
       </c>
       <c r="G968" s="2" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H968" s="2" t="inlineStr">
         <is>
@@ -38183,7 +38183,7 @@
       </c>
       <c r="I968" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -38291,7 +38291,7 @@
         </is>
       </c>
       <c r="G971" s="2" t="n">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="H971" s="2" t="inlineStr">
         <is>
@@ -38599,11 +38599,11 @@
       <c r="E979" s="2" t="inlineStr"/>
       <c r="F979" s="2" t="inlineStr">
         <is>
-          <t>24.00</t>
+          <t>25.50</t>
         </is>
       </c>
       <c r="G979" s="2" t="n">
-        <v>456</v>
+        <v>756</v>
       </c>
       <c r="H979" s="2" t="inlineStr">
         <is>
@@ -38642,7 +38642,7 @@
         </is>
       </c>
       <c r="G980" s="2" t="n">
-        <v>519</v>
+        <v>509</v>
       </c>
       <c r="H980" s="2" t="inlineStr">
         <is>
@@ -39028,11 +39028,11 @@
       <c r="E990" s="2" t="inlineStr"/>
       <c r="F990" s="2" t="inlineStr">
         <is>
-          <t>21.00</t>
+          <t>19.50</t>
         </is>
       </c>
       <c r="G990" s="2" t="n">
-        <v>422</v>
+        <v>807</v>
       </c>
       <c r="H990" s="2" t="inlineStr">
         <is>
@@ -39067,11 +39067,11 @@
       <c r="E991" s="2" t="inlineStr"/>
       <c r="F991" s="2" t="inlineStr">
         <is>
-          <t>21.00</t>
+          <t>19.50</t>
         </is>
       </c>
       <c r="G991" s="2" t="n">
-        <v>8</v>
+        <v>407</v>
       </c>
       <c r="H991" s="2" t="inlineStr">
         <is>
@@ -39110,7 +39110,7 @@
         </is>
       </c>
       <c r="G992" s="2" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H992" s="2" t="inlineStr">
         <is>
@@ -39422,7 +39422,7 @@
         </is>
       </c>
       <c r="G1000" s="2" t="n">
-        <v>2</v>
+        <v>101</v>
       </c>
       <c r="H1000" s="2" t="inlineStr">
         <is>
@@ -39500,7 +39500,7 @@
         </is>
       </c>
       <c r="G1002" s="2" t="n">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="H1002" s="2" t="inlineStr">
         <is>
@@ -39578,7 +39578,7 @@
         </is>
       </c>
       <c r="G1004" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="H1004" s="2" t="inlineStr">
         <is>
@@ -39617,7 +39617,7 @@
         </is>
       </c>
       <c r="G1005" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H1005" s="2" t="inlineStr">
         <is>
@@ -39695,7 +39695,7 @@
         </is>
       </c>
       <c r="G1007" s="2" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="H1007" s="2" t="inlineStr">
         <is>
@@ -39773,7 +39773,7 @@
         </is>
       </c>
       <c r="G1009" s="2" t="n">
-        <v>278</v>
+        <v>55</v>
       </c>
       <c r="H1009" s="2" t="inlineStr">
         <is>
@@ -39812,7 +39812,7 @@
         </is>
       </c>
       <c r="G1010" s="2" t="n">
-        <v>277</v>
+        <v>65</v>
       </c>
       <c r="H1010" s="2" t="inlineStr">
         <is>
@@ -39851,7 +39851,7 @@
         </is>
       </c>
       <c r="G1011" s="2" t="n">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="H1011" s="2" t="inlineStr">
         <is>
@@ -39890,7 +39890,7 @@
         </is>
       </c>
       <c r="G1012" s="2" t="n">
-        <v>1256</v>
+        <v>1251</v>
       </c>
       <c r="H1012" s="2" t="inlineStr">
         <is>
@@ -39929,7 +39929,7 @@
         </is>
       </c>
       <c r="G1013" s="2" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H1013" s="2" t="inlineStr">
         <is>
@@ -39968,7 +39968,7 @@
         </is>
       </c>
       <c r="G1014" s="2" t="n">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="H1014" s="2" t="inlineStr">
         <is>
@@ -40124,7 +40124,7 @@
         </is>
       </c>
       <c r="G1018" s="2" t="n">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H1018" s="2" t="inlineStr">
         <is>
@@ -40163,7 +40163,7 @@
         </is>
       </c>
       <c r="G1019" s="2" t="n">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="H1019" s="2" t="inlineStr">
         <is>
@@ -40280,7 +40280,7 @@
         </is>
       </c>
       <c r="G1022" s="2" t="n">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="H1022" s="2" t="inlineStr">
         <is>
@@ -40319,7 +40319,7 @@
         </is>
       </c>
       <c r="G1023" s="2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H1023" s="2" t="inlineStr">
         <is>
@@ -40358,7 +40358,7 @@
         </is>
       </c>
       <c r="G1024" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H1024" s="2" t="inlineStr">
         <is>
@@ -40397,7 +40397,7 @@
         </is>
       </c>
       <c r="G1025" s="2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H1025" s="2" t="inlineStr">
         <is>
@@ -40436,7 +40436,7 @@
         </is>
       </c>
       <c r="G1026" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H1026" s="2" t="inlineStr">
         <is>
@@ -40553,7 +40553,7 @@
         </is>
       </c>
       <c r="G1029" s="2" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H1029" s="2" t="inlineStr">
         <is>
@@ -40592,7 +40592,7 @@
         </is>
       </c>
       <c r="G1030" s="2" t="n">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="H1030" s="2" t="inlineStr">
         <is>
@@ -40631,7 +40631,7 @@
         </is>
       </c>
       <c r="G1031" s="2" t="n">
-        <v>571</v>
+        <v>527</v>
       </c>
       <c r="H1031" s="2" t="inlineStr">
         <is>
@@ -40670,7 +40670,7 @@
         </is>
       </c>
       <c r="G1032" s="2" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H1032" s="2" t="inlineStr">
         <is>
@@ -40709,7 +40709,7 @@
         </is>
       </c>
       <c r="G1033" s="2" t="n">
-        <v>84</v>
+        <v>62</v>
       </c>
       <c r="H1033" s="2" t="inlineStr">
         <is>
@@ -40748,7 +40748,7 @@
         </is>
       </c>
       <c r="G1034" s="2" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="H1034" s="2" t="inlineStr">
         <is>
@@ -40826,7 +40826,7 @@
         </is>
       </c>
       <c r="G1036" s="2" t="n">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="H1036" s="2" t="inlineStr">
         <is>
@@ -41021,7 +41021,7 @@
         </is>
       </c>
       <c r="G1041" s="2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H1041" s="2" t="inlineStr">
         <is>
@@ -41060,7 +41060,7 @@
         </is>
       </c>
       <c r="G1042" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H1042" s="2" t="inlineStr">
         <is>
@@ -41177,7 +41177,7 @@
         </is>
       </c>
       <c r="G1045" s="2" t="n">
-        <v>475</v>
+        <v>372</v>
       </c>
       <c r="H1045" s="2" t="inlineStr">
         <is>
@@ -41216,7 +41216,7 @@
         </is>
       </c>
       <c r="G1046" s="2" t="n">
-        <v>266</v>
+        <v>164</v>
       </c>
       <c r="H1046" s="2" t="inlineStr">
         <is>
@@ -41255,7 +41255,7 @@
         </is>
       </c>
       <c r="G1047" s="2" t="n">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="H1047" s="2" t="inlineStr">
         <is>
@@ -41450,7 +41450,7 @@
         </is>
       </c>
       <c r="G1052" s="2" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H1052" s="2" t="inlineStr">
         <is>
@@ -41996,7 +41996,7 @@
         </is>
       </c>
       <c r="G1066" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H1066" s="2" t="inlineStr">
         <is>
@@ -42035,7 +42035,7 @@
         </is>
       </c>
       <c r="G1067" s="2" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H1067" s="2" t="inlineStr">
         <is>
@@ -42503,7 +42503,7 @@
         </is>
       </c>
       <c r="G1079" s="2" t="n">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="H1079" s="2" t="inlineStr">
         <is>
@@ -42581,7 +42581,7 @@
         </is>
       </c>
       <c r="G1081" s="2" t="n">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="H1081" s="2" t="inlineStr">
         <is>
@@ -43322,7 +43322,7 @@
         </is>
       </c>
       <c r="G1100" s="2" t="n">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="H1100" s="2" t="inlineStr">
         <is>
@@ -43361,7 +43361,7 @@
         </is>
       </c>
       <c r="G1101" s="2" t="n">
-        <v>571</v>
+        <v>1159</v>
       </c>
       <c r="H1101" s="2" t="inlineStr">
         <is>
@@ -43400,7 +43400,7 @@
         </is>
       </c>
       <c r="G1102" s="2" t="n">
-        <v>938</v>
+        <v>925</v>
       </c>
       <c r="H1102" s="2" t="inlineStr">
         <is>
@@ -43595,7 +43595,7 @@
         </is>
       </c>
       <c r="G1107" s="2" t="n">
-        <v>227</v>
+        <v>424</v>
       </c>
       <c r="H1107" s="2" t="inlineStr">
         <is>
@@ -43946,7 +43946,7 @@
         </is>
       </c>
       <c r="G1116" s="2" t="n">
-        <v>321</v>
+        <v>288</v>
       </c>
       <c r="H1116" s="2" t="inlineStr">
         <is>
@@ -44219,7 +44219,7 @@
         </is>
       </c>
       <c r="G1123" s="2" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="H1123" s="2" t="inlineStr">
         <is>
@@ -44492,7 +44492,7 @@
         </is>
       </c>
       <c r="G1130" s="2" t="n">
-        <v>402</v>
+        <v>388</v>
       </c>
       <c r="H1130" s="2" t="inlineStr">
         <is>
@@ -44609,7 +44609,7 @@
         </is>
       </c>
       <c r="G1133" s="2" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="H1133" s="2" t="inlineStr">
         <is>
@@ -44687,7 +44687,7 @@
         </is>
       </c>
       <c r="G1135" s="2" t="n">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="H1135" s="2" t="inlineStr">
         <is>
@@ -44765,7 +44765,7 @@
         </is>
       </c>
       <c r="G1137" s="2" t="n">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="H1137" s="2" t="inlineStr">
         <is>
@@ -45857,7 +45857,7 @@
         </is>
       </c>
       <c r="G1165" s="2" t="n">
-        <v>875</v>
+        <v>870</v>
       </c>
       <c r="H1165" s="2" t="inlineStr">
         <is>
@@ -45896,7 +45896,7 @@
         </is>
       </c>
       <c r="G1166" s="2" t="n">
-        <v>1055</v>
+        <v>1036</v>
       </c>
       <c r="H1166" s="2" t="inlineStr">
         <is>
@@ -45974,7 +45974,7 @@
         </is>
       </c>
       <c r="G1168" s="2" t="n">
-        <v>0</v>
+        <v>280</v>
       </c>
       <c r="H1168" s="2" t="inlineStr">
         <is>
@@ -45983,7 +45983,7 @@
       </c>
       <c r="I1168" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -46013,7 +46013,7 @@
         </is>
       </c>
       <c r="G1169" s="2" t="n">
-        <v>346</v>
+        <v>456</v>
       </c>
       <c r="H1169" s="2" t="inlineStr">
         <is>
@@ -46052,7 +46052,7 @@
         </is>
       </c>
       <c r="G1170" s="2" t="n">
-        <v>472</v>
+        <v>457</v>
       </c>
       <c r="H1170" s="2" t="inlineStr">
         <is>
@@ -46091,7 +46091,7 @@
         </is>
       </c>
       <c r="G1171" s="2" t="n">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="H1171" s="2" t="inlineStr">
         <is>
@@ -46130,7 +46130,7 @@
         </is>
       </c>
       <c r="G1172" s="2" t="n">
-        <v>1050</v>
+        <v>1014</v>
       </c>
       <c r="H1172" s="2" t="inlineStr">
         <is>
@@ -46481,7 +46481,7 @@
         </is>
       </c>
       <c r="G1181" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H1181" s="2" t="inlineStr">
         <is>
@@ -47144,7 +47144,7 @@
         </is>
       </c>
       <c r="G1198" s="2" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H1198" s="2" t="inlineStr">
         <is>
@@ -48236,7 +48236,7 @@
         </is>
       </c>
       <c r="G1226" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H1226" s="2" t="inlineStr">
         <is>
@@ -48938,7 +48938,7 @@
         </is>
       </c>
       <c r="G1244" s="2" t="n">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="H1244" s="2" t="inlineStr">
         <is>
@@ -49328,7 +49328,7 @@
         </is>
       </c>
       <c r="G1254" s="2" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="H1254" s="2" t="inlineStr">
         <is>
@@ -49367,7 +49367,7 @@
         </is>
       </c>
       <c r="G1255" s="2" t="n">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H1255" s="2" t="inlineStr">
         <is>
@@ -49406,7 +49406,7 @@
         </is>
       </c>
       <c r="G1256" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H1256" s="2" t="inlineStr">
         <is>
@@ -49484,7 +49484,7 @@
         </is>
       </c>
       <c r="G1258" s="2" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="H1258" s="2" t="inlineStr">
         <is>
@@ -49523,7 +49523,7 @@
         </is>
       </c>
       <c r="G1259" s="2" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H1259" s="2" t="inlineStr">
         <is>
@@ -49796,7 +49796,7 @@
         </is>
       </c>
       <c r="G1266" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H1266" s="2" t="inlineStr">
         <is>
@@ -50693,7 +50693,7 @@
         </is>
       </c>
       <c r="G1289" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H1289" s="2" t="inlineStr">
         <is>
@@ -50849,7 +50849,7 @@
         </is>
       </c>
       <c r="G1293" s="2" t="n">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="H1293" s="2" t="inlineStr">
         <is>
@@ -51200,7 +51200,7 @@
         </is>
       </c>
       <c r="G1302" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H1302" s="2" t="inlineStr">
         <is>
@@ -51317,7 +51317,7 @@
         </is>
       </c>
       <c r="G1305" s="2" t="n">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H1305" s="2" t="inlineStr">
         <is>
@@ -52218,7 +52218,7 @@
       </c>
       <c r="H1328" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I1328" s="2" t="inlineStr">
@@ -52526,7 +52526,7 @@
         </is>
       </c>
       <c r="G1336" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H1336" s="2" t="inlineStr">
         <is>
@@ -52760,7 +52760,7 @@
         </is>
       </c>
       <c r="G1342" s="2" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H1342" s="2" t="inlineStr">
         <is>
@@ -52877,7 +52877,7 @@
         </is>
       </c>
       <c r="G1345" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="H1345" s="2" t="inlineStr">
         <is>
@@ -52916,7 +52916,7 @@
         </is>
       </c>
       <c r="G1346" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H1346" s="2" t="inlineStr">
         <is>
@@ -53033,7 +53033,7 @@
         </is>
       </c>
       <c r="G1349" s="2" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="H1349" s="2" t="inlineStr">
         <is>
@@ -53150,7 +53150,7 @@
         </is>
       </c>
       <c r="G1352" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H1352" s="2" t="inlineStr">
         <is>
@@ -53462,7 +53462,7 @@
         </is>
       </c>
       <c r="G1360" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H1360" s="2" t="inlineStr">
         <is>
@@ -53501,7 +53501,7 @@
         </is>
       </c>
       <c r="G1361" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1361" s="2" t="inlineStr">
         <is>
@@ -53579,7 +53579,7 @@
         </is>
       </c>
       <c r="G1363" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H1363" s="2" t="inlineStr">
         <is>
@@ -53657,7 +53657,7 @@
         </is>
       </c>
       <c r="G1365" s="2" t="n">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="H1365" s="2" t="inlineStr">
         <is>
@@ -53696,7 +53696,7 @@
         </is>
       </c>
       <c r="G1366" s="2" t="n">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="H1366" s="2" t="inlineStr">
         <is>
@@ -53735,7 +53735,7 @@
         </is>
       </c>
       <c r="G1367" s="2" t="n">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H1367" s="2" t="inlineStr">
         <is>
@@ -53774,7 +53774,7 @@
         </is>
       </c>
       <c r="G1368" s="2" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H1368" s="2" t="inlineStr">
         <is>
@@ -54008,7 +54008,7 @@
         </is>
       </c>
       <c r="G1374" s="2" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H1374" s="2" t="inlineStr">
         <is>
@@ -54164,7 +54164,7 @@
         </is>
       </c>
       <c r="G1378" s="2" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H1378" s="2" t="inlineStr">
         <is>
@@ -55330,11 +55330,11 @@
       <c r="E1408" s="2" t="inlineStr"/>
       <c r="F1408" s="2" t="inlineStr">
         <is>
-          <t>267.00</t>
+          <t>270.00</t>
         </is>
       </c>
       <c r="G1408" s="2" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="H1408" s="2" t="inlineStr">
         <is>
@@ -55373,7 +55373,7 @@
         </is>
       </c>
       <c r="G1409" s="2" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H1409" s="2" t="inlineStr">
         <is>
@@ -55412,7 +55412,7 @@
         </is>
       </c>
       <c r="G1410" s="2" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H1410" s="2" t="inlineStr">
         <is>
@@ -55646,7 +55646,7 @@
         </is>
       </c>
       <c r="G1416" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H1416" s="2" t="inlineStr">
         <is>
@@ -56578,11 +56578,11 @@
       <c r="E1440" s="2" t="inlineStr"/>
       <c r="F1440" s="2" t="inlineStr">
         <is>
-          <t>108.00</t>
+          <t>99.00</t>
         </is>
       </c>
       <c r="G1440" s="2" t="n">
-        <v>77</v>
+        <v>269</v>
       </c>
       <c r="H1440" s="2" t="inlineStr">
         <is>
@@ -56738,7 +56738,7 @@
         </is>
       </c>
       <c r="G1444" s="2" t="n">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="H1444" s="2" t="inlineStr">
         <is>
@@ -56812,11 +56812,11 @@
       <c r="E1446" s="2" t="inlineStr"/>
       <c r="F1446" s="2" t="inlineStr">
         <is>
-          <t>114.00</t>
+          <t>105.00</t>
         </is>
       </c>
       <c r="G1446" s="2" t="n">
-        <v>184</v>
+        <v>382</v>
       </c>
       <c r="H1446" s="2" t="inlineStr">
         <is>
@@ -57050,7 +57050,7 @@
         </is>
       </c>
       <c r="G1452" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H1452" s="2" t="inlineStr">
         <is>
@@ -57089,7 +57089,7 @@
         </is>
       </c>
       <c r="G1453" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H1453" s="2" t="inlineStr">
         <is>
@@ -57128,7 +57128,7 @@
         </is>
       </c>
       <c r="G1454" s="2" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="H1454" s="2" t="inlineStr">
         <is>
@@ -57167,7 +57167,7 @@
         </is>
       </c>
       <c r="G1455" s="2" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H1455" s="2" t="inlineStr">
         <is>
@@ -57206,7 +57206,7 @@
         </is>
       </c>
       <c r="G1456" s="2" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H1456" s="2" t="inlineStr">
         <is>
@@ -57245,7 +57245,7 @@
         </is>
       </c>
       <c r="G1457" s="2" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H1457" s="2" t="inlineStr">
         <is>
@@ -58493,7 +58493,7 @@
         </is>
       </c>
       <c r="G1489" s="2" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H1489" s="2" t="inlineStr">
         <is>
@@ -58532,7 +58532,7 @@
         </is>
       </c>
       <c r="G1490" s="2" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H1490" s="2" t="inlineStr">
         <is>
@@ -58961,7 +58961,7 @@
         </is>
       </c>
       <c r="G1501" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1501" s="2" t="inlineStr">
         <is>
@@ -58970,7 +58970,7 @@
       </c>
       <c r="I1501" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -59390,7 +59390,7 @@
         </is>
       </c>
       <c r="G1512" s="2" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H1512" s="2" t="inlineStr">
         <is>
@@ -59468,7 +59468,7 @@
         </is>
       </c>
       <c r="G1514" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H1514" s="2" t="inlineStr">
         <is>
@@ -60053,7 +60053,7 @@
         </is>
       </c>
       <c r="G1529" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H1529" s="2" t="inlineStr">
         <is>
@@ -60092,7 +60092,7 @@
         </is>
       </c>
       <c r="G1530" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H1530" s="2" t="inlineStr">
         <is>
@@ -60131,7 +60131,7 @@
         </is>
       </c>
       <c r="G1531" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1531" s="2" t="inlineStr">
         <is>
@@ -60140,7 +60140,7 @@
       </c>
       <c r="I1531" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -60170,7 +60170,7 @@
         </is>
       </c>
       <c r="G1532" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H1532" s="2" t="inlineStr">
         <is>
@@ -60209,7 +60209,7 @@
         </is>
       </c>
       <c r="G1533" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1533" s="2" t="inlineStr">
         <is>
@@ -60218,7 +60218,7 @@
       </c>
       <c r="I1533" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -60443,7 +60443,7 @@
         </is>
       </c>
       <c r="G1539" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H1539" s="2" t="inlineStr">
         <is>
@@ -60638,7 +60638,7 @@
         </is>
       </c>
       <c r="G1544" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H1544" s="2" t="inlineStr">
         <is>
@@ -60755,7 +60755,7 @@
         </is>
       </c>
       <c r="G1547" s="2" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="H1547" s="2" t="inlineStr">
         <is>
@@ -60794,7 +60794,7 @@
         </is>
       </c>
       <c r="G1548" s="2" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="H1548" s="2" t="inlineStr">
         <is>
@@ -60872,7 +60872,7 @@
         </is>
       </c>
       <c r="G1550" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H1550" s="2" t="inlineStr">
         <is>
@@ -60989,7 +60989,7 @@
         </is>
       </c>
       <c r="G1553" s="2" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="H1553" s="2" t="inlineStr">
         <is>
@@ -61028,7 +61028,7 @@
         </is>
       </c>
       <c r="G1554" s="2" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="H1554" s="2" t="inlineStr">
         <is>
@@ -61067,7 +61067,7 @@
         </is>
       </c>
       <c r="G1555" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H1555" s="2" t="inlineStr">
         <is>
@@ -61076,7 +61076,7 @@
       </c>
       <c r="I1555" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -61106,7 +61106,7 @@
         </is>
       </c>
       <c r="G1556" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H1556" s="2" t="inlineStr">
         <is>
@@ -61115,7 +61115,7 @@
       </c>
       <c r="I1556" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -61145,7 +61145,7 @@
         </is>
       </c>
       <c r="G1557" s="2" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H1557" s="2" t="inlineStr">
         <is>
@@ -61223,7 +61223,7 @@
         </is>
       </c>
       <c r="G1559" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H1559" s="2" t="inlineStr">
         <is>
@@ -61262,7 +61262,7 @@
         </is>
       </c>
       <c r="G1560" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H1560" s="2" t="inlineStr">
         <is>
@@ -61301,7 +61301,7 @@
         </is>
       </c>
       <c r="G1561" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H1561" s="2" t="inlineStr">
         <is>
@@ -61691,7 +61691,7 @@
         </is>
       </c>
       <c r="G1571" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H1571" s="2" t="inlineStr">
         <is>
@@ -61730,7 +61730,7 @@
         </is>
       </c>
       <c r="G1572" s="2" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="H1572" s="2" t="inlineStr">
         <is>
@@ -61769,7 +61769,7 @@
         </is>
       </c>
       <c r="G1573" s="2" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H1573" s="2" t="inlineStr">
         <is>
@@ -61808,7 +61808,7 @@
         </is>
       </c>
       <c r="G1574" s="2" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H1574" s="2" t="inlineStr">
         <is>
@@ -62198,7 +62198,7 @@
         </is>
       </c>
       <c r="G1584" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H1584" s="2" t="inlineStr">
         <is>
@@ -62207,7 +62207,7 @@
       </c>
       <c r="I1584" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -62666,16 +62666,16 @@
         </is>
       </c>
       <c r="G1596" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H1596" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I1596" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -62709,7 +62709,7 @@
       </c>
       <c r="H1597" s="2" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>unlisted</t>
         </is>
       </c>
       <c r="I1597" s="2" t="inlineStr">
@@ -62783,7 +62783,7 @@
         </is>
       </c>
       <c r="G1599" s="2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H1599" s="2" t="inlineStr">
         <is>
@@ -62939,7 +62939,7 @@
         </is>
       </c>
       <c r="G1603" s="2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H1603" s="2" t="inlineStr">
         <is>
@@ -62978,7 +62978,7 @@
         </is>
       </c>
       <c r="G1604" s="2" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H1604" s="2" t="inlineStr">
         <is>
@@ -63056,7 +63056,7 @@
         </is>
       </c>
       <c r="G1606" s="2" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H1606" s="2" t="inlineStr">
         <is>
@@ -63095,7 +63095,7 @@
         </is>
       </c>
       <c r="G1607" s="2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H1607" s="2" t="inlineStr">
         <is>
@@ -63543,7 +63543,7 @@
       </c>
       <c r="B1619" s="2" t="inlineStr">
         <is>
-          <t>Proyector Profesional Android 4k Hd Wifi Smart Tv Portatil Bluetooth 110v/220v</t>
+          <t>Proyector Profesional Android 4k Hd Wifi Smart Tv Portatil Bluetooth 110v/220v HY300</t>
         </is>
       </c>
       <c r="C1619" s="2" t="inlineStr">
@@ -64031,7 +64031,7 @@
         </is>
       </c>
       <c r="G1631" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H1631" s="2" t="inlineStr">
         <is>
@@ -64265,7 +64265,7 @@
         </is>
       </c>
       <c r="G1637" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H1637" s="2" t="inlineStr">
         <is>
@@ -65006,7 +65006,7 @@
         </is>
       </c>
       <c r="G1656" s="2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H1656" s="2" t="inlineStr">
         <is>
@@ -65552,7 +65552,7 @@
         </is>
       </c>
       <c r="G1670" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H1670" s="2" t="inlineStr">
         <is>
@@ -65591,7 +65591,7 @@
         </is>
       </c>
       <c r="G1671" s="2" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H1671" s="2" t="inlineStr">
         <is>
@@ -68165,7 +68165,7 @@
         </is>
       </c>
       <c r="G1737" s="2" t="n">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="H1737" s="2" t="inlineStr">
         <is>
@@ -68204,7 +68204,7 @@
         </is>
       </c>
       <c r="G1738" s="2" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="H1738" s="2" t="inlineStr">
         <is>
@@ -68243,7 +68243,7 @@
         </is>
       </c>
       <c r="G1739" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H1739" s="2" t="inlineStr">
         <is>
@@ -68252,7 +68252,7 @@
       </c>
       <c r="I1739" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -68282,7 +68282,7 @@
         </is>
       </c>
       <c r="G1740" s="2" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="H1740" s="2" t="inlineStr">
         <is>
@@ -68438,7 +68438,7 @@
         </is>
       </c>
       <c r="G1744" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H1744" s="2" t="inlineStr">
         <is>
@@ -68477,7 +68477,7 @@
         </is>
       </c>
       <c r="G1745" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H1745" s="2" t="inlineStr">
         <is>
@@ -68789,7 +68789,7 @@
         </is>
       </c>
       <c r="G1753" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H1753" s="2" t="inlineStr">
         <is>
@@ -70349,7 +70349,7 @@
         </is>
       </c>
       <c r="G1793" s="2" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H1793" s="2" t="inlineStr">
         <is>
@@ -70388,7 +70388,7 @@
         </is>
       </c>
       <c r="G1794" s="2" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H1794" s="2" t="inlineStr">
         <is>
@@ -70427,7 +70427,7 @@
         </is>
       </c>
       <c r="G1795" s="2" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="H1795" s="2" t="inlineStr">
         <is>
@@ -70466,7 +70466,7 @@
         </is>
       </c>
       <c r="G1796" s="2" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H1796" s="2" t="inlineStr">
         <is>
@@ -70583,7 +70583,7 @@
         </is>
       </c>
       <c r="G1799" s="2" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H1799" s="2" t="inlineStr">
         <is>
@@ -70622,7 +70622,7 @@
         </is>
       </c>
       <c r="G1800" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H1800" s="2" t="inlineStr">
         <is>
@@ -70739,7 +70739,7 @@
         </is>
       </c>
       <c r="G1803" s="2" t="n">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="H1803" s="2" t="inlineStr">
         <is>
@@ -70778,7 +70778,7 @@
         </is>
       </c>
       <c r="G1804" s="2" t="n">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="H1804" s="2" t="inlineStr">
         <is>
@@ -70817,7 +70817,7 @@
         </is>
       </c>
       <c r="G1805" s="2" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="H1805" s="2" t="inlineStr">
         <is>
@@ -70856,7 +70856,7 @@
         </is>
       </c>
       <c r="G1806" s="2" t="n">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="H1806" s="2" t="inlineStr">
         <is>
@@ -70895,7 +70895,7 @@
         </is>
       </c>
       <c r="G1807" s="2" t="n">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="H1807" s="2" t="inlineStr">
         <is>
@@ -70973,7 +70973,7 @@
         </is>
       </c>
       <c r="G1809" s="2" t="n">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="H1809" s="2" t="inlineStr">
         <is>
@@ -71051,7 +71051,7 @@
         </is>
       </c>
       <c r="G1811" s="2" t="n">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="H1811" s="2" t="inlineStr">
         <is>
@@ -71090,7 +71090,7 @@
         </is>
       </c>
       <c r="G1812" s="2" t="n">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="H1812" s="2" t="inlineStr">
         <is>
@@ -71207,7 +71207,7 @@
         </is>
       </c>
       <c r="G1815" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H1815" s="2" t="inlineStr">
         <is>
@@ -71402,7 +71402,7 @@
         </is>
       </c>
       <c r="G1820" s="2" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="H1820" s="2" t="inlineStr">
         <is>
@@ -73274,7 +73274,7 @@
         </is>
       </c>
       <c r="G1868" s="2" t="n">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="H1868" s="2" t="inlineStr">
         <is>
@@ -73313,7 +73313,7 @@
         </is>
       </c>
       <c r="G1869" s="2" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H1869" s="2" t="inlineStr">
         <is>
@@ -73391,7 +73391,7 @@
         </is>
       </c>
       <c r="G1871" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="H1871" s="2" t="inlineStr">
         <is>
@@ -73469,7 +73469,7 @@
         </is>
       </c>
       <c r="G1873" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H1873" s="2" t="inlineStr">
         <is>
@@ -73547,7 +73547,7 @@
         </is>
       </c>
       <c r="G1875" s="2" t="n">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="H1875" s="2" t="inlineStr">
         <is>
@@ -73664,7 +73664,7 @@
         </is>
       </c>
       <c r="G1878" s="2" t="n">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H1878" s="2" t="inlineStr">
         <is>
@@ -73820,7 +73820,7 @@
         </is>
       </c>
       <c r="G1882" s="2" t="n">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="H1882" s="2" t="inlineStr">
         <is>
@@ -73859,7 +73859,7 @@
         </is>
       </c>
       <c r="G1883" s="2" t="n">
-        <v>323</v>
+        <v>261</v>
       </c>
       <c r="H1883" s="2" t="inlineStr">
         <is>
@@ -73976,7 +73976,7 @@
         </is>
       </c>
       <c r="G1886" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H1886" s="2" t="inlineStr">
         <is>
@@ -74015,7 +74015,7 @@
         </is>
       </c>
       <c r="G1887" s="2" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H1887" s="2" t="inlineStr">
         <is>
@@ -74210,7 +74210,7 @@
         </is>
       </c>
       <c r="G1892" s="2" t="n">
-        <v>454</v>
+        <v>352</v>
       </c>
       <c r="H1892" s="2" t="inlineStr">
         <is>
@@ -74717,12 +74717,12 @@
       </c>
       <c r="H1905" s="2" t="inlineStr">
         <is>
-          <t>unlisted</t>
+          <t>active</t>
         </is>
       </c>
       <c r="I1905" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -74752,7 +74752,7 @@
         </is>
       </c>
       <c r="G1906" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H1906" s="2" t="inlineStr">
         <is>
@@ -74761,7 +74761,7 @@
       </c>
       <c r="I1906" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>
@@ -75181,7 +75181,7 @@
         </is>
       </c>
       <c r="G1917" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H1917" s="2" t="inlineStr">
         <is>
@@ -75532,7 +75532,7 @@
         </is>
       </c>
       <c r="G1926" s="2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H1926" s="2" t="inlineStr">
         <is>
@@ -75610,7 +75610,7 @@
         </is>
       </c>
       <c r="G1928" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H1928" s="2" t="inlineStr">
         <is>
@@ -75844,7 +75844,7 @@
         </is>
       </c>
       <c r="G1934" s="2" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="H1934" s="2" t="inlineStr">
         <is>

</xml_diff>